<commit_message>
VistaWish Implementada con kpi comparando wishlist con entas en dia y semana 1, logica de informe detallado actualizado con los datos recopilados de vistaWish
</commit_message>
<xml_diff>
--- a/app/assets/steam_db.xlsx
+++ b/app/assets/steam_db.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="110">
   <si>
     <t>ID</t>
   </si>
@@ -343,6 +343,12 @@
   </si>
   <si>
     <t>Final Frontier</t>
+  </si>
+  <si>
+    <t>Carrillo es gay</t>
+  </si>
+  <si>
+    <t>aventura</t>
   </si>
 </sst>
 </file>
@@ -617,10 +623,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,7 +658,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -684,7 +690,7 @@
         <v>12300</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -716,7 +722,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -748,7 +754,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -780,7 +786,7 @@
         <v>28000</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -812,7 +818,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -844,7 +850,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -876,7 +882,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -908,7 +914,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -940,7 +946,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -972,7 +978,7 @@
         <v>9800</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1004,7 +1010,7 @@
         <v>2900</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1036,7 +1042,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1068,7 +1074,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1100,7 +1106,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1132,7 +1138,7 @@
         <v>3200</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1164,7 +1170,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1196,7 +1202,7 @@
         <v>8100</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1228,7 +1234,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1260,7 +1266,7 @@
         <v>21500</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1292,7 +1298,7 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1324,7 +1330,7 @@
         <v>9400</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1356,7 +1362,7 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1388,7 +1394,7 @@
         <v>5800</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1420,7 +1426,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1452,7 +1458,7 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1484,7 +1490,7 @@
         <v>1850</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1516,7 +1522,7 @@
         <v>13200</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1549,7 +1555,7 @@
       </c>
       <c r="M29" s="2"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1581,7 +1587,7 @@
         <v>7600</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1613,7 +1619,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1645,7 +1651,7 @@
         <v>4100</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1677,7 +1683,7 @@
         <v>3600</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1709,7 +1715,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1741,7 +1747,7 @@
         <v>22100</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1773,7 +1779,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1805,7 +1811,7 @@
         <v>6400</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1837,7 +1843,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1869,7 +1875,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -1901,7 +1907,7 @@
         <v>15900</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -1933,7 +1939,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -1965,7 +1971,7 @@
         <v>54000</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -1997,7 +2003,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -2029,7 +2035,7 @@
         <v>2150</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -2061,7 +2067,7 @@
         <v>10200</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -2093,7 +2099,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -2125,7 +2131,7 @@
         <v>25600</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -2157,7 +2163,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -2189,7 +2195,7 @@
         <v>3100</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -2221,7 +2227,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -2252,6 +2258,44 @@
       <c r="J51" s="1">
         <v>31000</v>
       </c>
+    </row>
+    <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="1">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D52" s="1">
+        <v>2020</v>
+      </c>
+      <c r="E52" s="1">
+        <v>3</v>
+      </c>
+      <c r="F52" s="1">
+        <v>10</v>
+      </c>
+      <c r="G52" s="1">
+        <v>2</v>
+      </c>
+      <c r="H52" s="1">
+        <v>3</v>
+      </c>
+      <c r="I52" s="1">
+        <v>4</v>
+      </c>
+      <c r="J52" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K54" s="2"/>
+    </row>
+    <row r="58" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E58" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>